<commit_message>
autopilot: drive to west successful completed
</commit_message>
<xml_diff>
--- a/sectoren vorlage.xlsx
+++ b/sectoren vorlage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nutzer\Documents\Java\SpringBoot3\ocean-explorer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACE178A-42C5-47A5-90A4-365A0D9438E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59119F86-5DBE-4374-BA23-25AFD395F238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13845" yWindow="0" windowWidth="13845" windowHeight="16200" firstSheet="2" activeTab="5" xr2:uid="{CE7404B4-C4A0-4B6E-9CA3-B25732518FF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="27930" windowHeight="16440" firstSheet="2" activeTab="4" xr2:uid="{CE7404B4-C4A0-4B6E-9CA3-B25732518FF2}"/>
   </bookViews>
   <sheets>
     <sheet name="do not delete" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
git ignore file erstellt
</commit_message>
<xml_diff>
--- a/sectoren vorlage.xlsx
+++ b/sectoren vorlage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nutzer\Documents\Java\SpringBoot3\ocean-explorer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59119F86-5DBE-4374-BA23-25AFD395F238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B5852D-14F5-485C-89B5-382233476B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="27930" windowHeight="16440" firstSheet="2" activeTab="4" xr2:uid="{CE7404B4-C4A0-4B6E-9CA3-B25732518FF2}"/>
   </bookViews>
@@ -129,6 +129,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -271,17 +274,15 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -635,31 +636,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="22" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="22" t="s">
+      <c r="E1" s="24"/>
+      <c r="F1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="22" t="s">
+      <c r="G1" s="24"/>
+      <c r="H1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="23"/>
+      <c r="I1" s="24"/>
       <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="K1" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="23"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="23"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="24"/>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -695,13 +696,13 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="24">
         <v>6</v>
       </c>
-      <c r="C3" s="23">
+      <c r="C3" s="24">
         <v>12</v>
       </c>
       <c r="D3" s="3">
@@ -736,9 +737,9 @@
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
       <c r="D4" s="3">
         <f>K3</f>
         <v>-1</v>
@@ -774,9 +775,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
       <c r="D5" s="3">
         <f t="shared" ref="D5:D25" si="0">K4</f>
         <v>-1</v>
@@ -812,9 +813,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -850,9 +851,9 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
       <c r="D7" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -882,13 +883,13 @@
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="24">
         <v>3</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="24">
         <v>6</v>
       </c>
       <c r="D9" s="3">
@@ -922,9 +923,9 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
       <c r="D10" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -960,9 +961,9 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -998,9 +999,9 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -1036,9 +1037,9 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -1074,9 +1075,9 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
       <c r="D14" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -1106,13 +1107,13 @@
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="24">
         <v>11</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="24">
         <v>7</v>
       </c>
       <c r="D16" s="3">
@@ -1146,9 +1147,9 @@
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1184,9 +1185,9 @@
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1222,9 +1223,9 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
       <c r="D19" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1254,13 +1255,13 @@
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="23">
+      <c r="B21" s="24">
         <v>12</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="24">
         <v>10</v>
       </c>
       <c r="D21" s="3">
@@ -1295,9 +1296,9 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
       <c r="D22" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1333,9 +1334,9 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
       <c r="D23" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1371,9 +1372,9 @@
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
       <c r="D24" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1409,9 +1410,9 @@
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
       <c r="D25" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -1439,6 +1440,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="H1:I1"/>
     <mergeCell ref="C21:C25"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="B3:B7"/>
@@ -1452,11 +1458,6 @@
     <mergeCell ref="C16:C19"/>
     <mergeCell ref="A21:A25"/>
     <mergeCell ref="B21:B25"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="H1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1510,15 +1511,15 @@
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B2" s="7"/>
@@ -1536,9 +1537,9 @@
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="AA2" s="23"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="AA2" s="24"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
@@ -1559,9 +1560,9 @@
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
-      <c r="R3" s="23"/>
-      <c r="S3" s="23"/>
-      <c r="AA3" s="23"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
+      <c r="AA3" s="24"/>
       <c r="AB3" s="12"/>
       <c r="AC3" s="12"/>
       <c r="AD3" s="12"/>
@@ -1587,9 +1588,9 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="AA4" s="23"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="AA4" s="24"/>
       <c r="AB4" s="12"/>
       <c r="AC4" s="12"/>
       <c r="AD4" s="12"/>
@@ -1615,9 +1616,9 @@
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
-      <c r="R5" s="23"/>
-      <c r="S5" s="23"/>
-      <c r="AA5" s="23"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="AA5" s="24"/>
       <c r="AB5" s="11"/>
       <c r="AC5" s="11"/>
       <c r="AD5" s="11"/>
@@ -1643,9 +1644,9 @@
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="23"/>
-      <c r="AA6" s="23"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="AA6" s="24"/>
       <c r="AB6" s="12"/>
       <c r="AC6" s="12"/>
       <c r="AD6" s="12"/>
@@ -1671,9 +1672,9 @@
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="23"/>
-      <c r="AA7" s="23"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="AA7" s="24"/>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
@@ -1694,9 +1695,9 @@
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
-      <c r="R8" s="23"/>
-      <c r="S8" s="23"/>
-      <c r="AA8" s="23"/>
+      <c r="R8" s="24"/>
+      <c r="S8" s="24"/>
+      <c r="AA8" s="24"/>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
@@ -1717,9 +1718,9 @@
       <c r="N9" s="7"/>
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
-      <c r="R9" s="23"/>
-      <c r="S9" s="23"/>
-      <c r="AA9" s="23"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="24"/>
+      <c r="AA9" s="24"/>
       <c r="AB9" s="11"/>
       <c r="AC9" s="11"/>
       <c r="AD9" s="11"/>
@@ -1745,9 +1746,9 @@
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
-      <c r="R10" s="23"/>
-      <c r="S10" s="23"/>
-      <c r="AA10" s="23"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="24"/>
+      <c r="AA10" s="24"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
@@ -1768,9 +1769,9 @@
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
-      <c r="R11" s="23"/>
-      <c r="S11" s="23"/>
-      <c r="AA11" s="23"/>
+      <c r="R11" s="24"/>
+      <c r="S11" s="24"/>
+      <c r="AA11" s="24"/>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
@@ -1791,9 +1792,9 @@
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
-      <c r="R12" s="23"/>
-      <c r="S12" s="23"/>
-      <c r="AA12" s="23"/>
+      <c r="R12" s="24"/>
+      <c r="S12" s="24"/>
+      <c r="AA12" s="24"/>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
@@ -1814,9 +1815,9 @@
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
-      <c r="R13" s="23"/>
-      <c r="S13" s="23"/>
-      <c r="AA13" s="23"/>
+      <c r="R13" s="24"/>
+      <c r="S13" s="24"/>
+      <c r="AA13" s="24"/>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
@@ -1837,9 +1838,9 @@
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="23"/>
-      <c r="AA14" s="23"/>
+      <c r="R14" s="24"/>
+      <c r="S14" s="24"/>
+      <c r="AA14" s="24"/>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
@@ -1860,9 +1861,9 @@
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
-      <c r="R15" s="23"/>
-      <c r="S15" s="23"/>
-      <c r="AA15" s="23"/>
+      <c r="R15" s="24"/>
+      <c r="S15" s="24"/>
+      <c r="AA15" s="24"/>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
@@ -1969,31 +1970,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="22" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="22" t="s">
+      <c r="E1" s="24"/>
+      <c r="F1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="22" t="s">
+      <c r="G1" s="24"/>
+      <c r="H1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="23"/>
+      <c r="I1" s="24"/>
       <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="K1" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="23"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="23"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="24"/>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2029,13 +2030,13 @@
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="24">
         <v>5</v>
       </c>
-      <c r="C3" s="23">
+      <c r="C3" s="24">
         <v>9</v>
       </c>
       <c r="D3" s="3">
@@ -2070,9 +2071,9 @@
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
       <c r="D4" s="3">
         <f>K3</f>
         <v>-1</v>
@@ -2108,9 +2109,9 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
       <c r="D5" s="3">
         <f t="shared" ref="D5:E25" si="0">K4</f>
         <v>-1</v>
@@ -2146,9 +2147,9 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2184,9 +2185,9 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
       <c r="D7" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2216,13 +2217,13 @@
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="24">
         <v>3</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="24">
         <v>6</v>
       </c>
       <c r="D9" s="3">
@@ -2256,9 +2257,9 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
       <c r="D10" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2294,9 +2295,9 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2332,9 +2333,9 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2370,9 +2371,9 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2408,9 +2409,9 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
       <c r="D14" s="3">
         <f t="shared" si="0"/>
         <v>-1</v>
@@ -2440,13 +2441,13 @@
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="24">
         <v>11</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="24">
         <v>7</v>
       </c>
       <c r="D16" s="3">
@@ -2480,9 +2481,9 @@
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2518,9 +2519,9 @@
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2556,9 +2557,9 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
       <c r="D19" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2588,13 +2589,13 @@
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="23">
+      <c r="B21" s="24">
         <v>11</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="24">
         <v>13</v>
       </c>
       <c r="D21" s="3">
@@ -2629,9 +2630,9 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
       <c r="D22" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2667,9 +2668,9 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
       <c r="D23" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -2705,9 +2706,9 @@
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
       <c r="D24" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2743,9 +2744,9 @@
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
       <c r="D25" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2781,9 +2782,9 @@
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
       <c r="D26" s="3">
         <f>K25</f>
         <v>0</v>
@@ -2819,9 +2820,9 @@
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
       <c r="D27" s="3">
         <f t="shared" ref="D27:E27" si="12">K26</f>
         <v>0</v>
@@ -2849,24 +2850,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="B21:B27"/>
+    <mergeCell ref="C21:C27"/>
+    <mergeCell ref="A21:A27"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="A9:A14"/>
+    <mergeCell ref="B9:B14"/>
+    <mergeCell ref="C9:C14"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="K1:L1"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="B9:B14"/>
-    <mergeCell ref="C9:C14"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="B21:B27"/>
-    <mergeCell ref="C21:C27"/>
-    <mergeCell ref="A21:A27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2920,15 +2921,15 @@
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="24"/>
     </row>
     <row r="2" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B2" s="16"/>
@@ -2948,9 +2949,9 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="AC2" s="23"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="AC2" s="24"/>
     </row>
     <row r="3" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B3" s="16"/>
@@ -2970,9 +2971,9 @@
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="T3" s="23"/>
-      <c r="U3" s="23"/>
-      <c r="AC3" s="23"/>
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="AC3" s="24"/>
       <c r="AD3" s="12"/>
       <c r="AE3" s="12"/>
       <c r="AF3" s="12"/>
@@ -2997,9 +2998,9 @@
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="AC4" s="23"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="AC4" s="24"/>
       <c r="AD4" s="12"/>
       <c r="AE4" s="12"/>
       <c r="AF4" s="12"/>
@@ -3024,9 +3025,9 @@
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
-      <c r="T5" s="23"/>
-      <c r="U5" s="23"/>
-      <c r="AC5" s="23"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="AC5" s="24"/>
       <c r="AD5" s="11"/>
       <c r="AE5" s="11"/>
       <c r="AF5" s="11"/>
@@ -3051,9 +3052,9 @@
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="23"/>
-      <c r="AC6" s="23"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
+      <c r="AC6" s="24"/>
       <c r="AD6" s="12"/>
       <c r="AE6" s="12"/>
       <c r="AF6" s="12"/>
@@ -3078,9 +3079,9 @@
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
-      <c r="T7" s="23"/>
-      <c r="U7" s="23"/>
-      <c r="AC7" s="23"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
+      <c r="AC7" s="24"/>
     </row>
     <row r="8" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B8" s="16"/>
@@ -3100,9 +3101,9 @@
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
-      <c r="T8" s="23"/>
-      <c r="U8" s="23"/>
-      <c r="AC8" s="23"/>
+      <c r="T8" s="24"/>
+      <c r="U8" s="24"/>
+      <c r="AC8" s="24"/>
     </row>
     <row r="9" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B9" s="16"/>
@@ -3122,9 +3123,9 @@
       <c r="P9" s="13"/>
       <c r="Q9" s="7"/>
       <c r="R9" s="7"/>
-      <c r="T9" s="23"/>
-      <c r="U9" s="23"/>
-      <c r="AC9" s="23"/>
+      <c r="T9" s="24"/>
+      <c r="U9" s="24"/>
+      <c r="AC9" s="24"/>
       <c r="AD9" s="11"/>
       <c r="AE9" s="11"/>
       <c r="AF9" s="11"/>
@@ -3149,9 +3150,9 @@
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
       <c r="R10" s="7"/>
-      <c r="T10" s="23"/>
-      <c r="U10" s="23"/>
-      <c r="AC10" s="23"/>
+      <c r="T10" s="24"/>
+      <c r="U10" s="24"/>
+      <c r="AC10" s="24"/>
     </row>
     <row r="11" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B11" s="16"/>
@@ -3194,7 +3195,7 @@
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
     <col min="3" max="12" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.42578125" customWidth="1"/>
+    <col min="13" max="13" width="3.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="3.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3213,7 +3214,9 @@
       <c r="K2" s="19"/>
       <c r="L2" s="19"/>
       <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
+      <c r="N2" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
@@ -3232,8 +3235,12 @@
       <c r="J3" s="19"/>
       <c r="K3" s="19"/>
       <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
+      <c r="M3" s="26">
+        <v>2.6</v>
+      </c>
+      <c r="N3" s="19">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -3252,8 +3259,12 @@
       <c r="J4" s="19"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
+      <c r="M4" s="19">
+        <v>5</v>
+      </c>
+      <c r="N4" s="19">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
@@ -3307,7 +3318,7 @@
       <c r="E7" s="10"/>
       <c r="F7" s="7"/>
       <c r="G7" s="19"/>
-      <c r="H7" s="24"/>
+      <c r="H7" s="7"/>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
       <c r="K7" s="19"/>
@@ -3356,11 +3367,11 @@
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="19"/>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="7" t="s">
         <v>18</v>
       </c>
       <c r="H9" s="19"/>
-      <c r="I9" s="24" t="s">
+      <c r="I9" s="7" t="s">
         <v>18</v>
       </c>
       <c r="J9" s="19"/>
@@ -3411,11 +3422,11 @@
       <c r="F11" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="25" t="s">
+      <c r="G11" s="22" t="s">
         <v>17</v>
       </c>
       <c r="H11" s="19"/>
-      <c r="I11" s="25" t="s">
+      <c r="I11" s="22" t="s">
         <v>17</v>
       </c>
       <c r="J11" s="14" t="s">
@@ -3505,7 +3516,7 @@
       </c>
       <c r="G15" s="19"/>
       <c r="H15" s="19"/>
-      <c r="I15" s="25"/>
+      <c r="I15" s="22"/>
       <c r="J15" s="19"/>
       <c r="K15" s="10" t="s">
         <v>19</v>
@@ -3528,14 +3539,14 @@
         <v>24</v>
       </c>
       <c r="E16" s="7"/>
-      <c r="F16" s="25" t="s">
+      <c r="F16" s="22" t="s">
         <v>17</v>
       </c>
       <c r="G16" s="20" t="s">
         <v>18</v>
       </c>
       <c r="H16" s="19"/>
-      <c r="I16" s="25" t="s">
+      <c r="I16" s="22" t="s">
         <v>17</v>
       </c>
       <c r="J16" s="20" t="s">
@@ -3565,7 +3576,7 @@
         <v>19</v>
       </c>
       <c r="H17" s="19"/>
-      <c r="I17" s="25"/>
+      <c r="I17" s="22"/>
       <c r="J17" s="7" t="s">
         <v>20</v>
       </c>
@@ -3970,7 +3981,7 @@
       <c r="A5">
         <v>46</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="23" t="s">
         <v>17</v>
       </c>
       <c r="C5">

</xml_diff>